<commit_message>
feat: Bo sung Sheet 4 'Doi Soat Giam Gia & Thoi Han' (So sanh quy cach/model va danh gia hieu luc 12 thang)
</commit_message>
<xml_diff>
--- a/data/Bao_Cao_Tham_Dinh_Trinh_Lanh_Dao.xlsx
+++ b/data/Bao_Cao_Tham_Dinh_Trinh_Lanh_Dao.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Báo Cáo Tổng Hợp" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Danh Mục Chi Tiết" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Hồ Sơ Chứng Cứ &amp; Hình Ảnh" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Đối Soát Giảm Giá &amp; Thời Hạn" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,8 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="16">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0&quot;%&quot;"/>
+  </numFmts>
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -115,8 +118,26 @@
       <color rgb="0015803D"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00E0F2FE"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00FEF3C7"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -159,6 +180,22 @@
         <bgColor rgb="00CBD5E1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000369A1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0092400E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -186,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -340,6 +377,31 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7781,7 +7843,7 @@
     <row r="2">
       <c r="A2" s="39" t="inlineStr">
         <is>
-          <t>Hồ sơ: Mau_Bang_Du_Toan_13_Cot - Bản Mới-111 | Cập nhật: 18/09/2026 14:28</t>
+          <t>Hồ sơ: Mau_Bang_Du_Toan_13_Cot - Bản Mới-111 | Cập nhật: 18/09/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -21319,4 +21381,1861 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>BẢNG ĐỐI SOÁT QUY CÁCH KỸ THUẬT &amp; ĐÁNH GIÁ HIỆU LỰC THỜI GIAN CÁC MỤC GIẢM GIÁ DỰ TOÁN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>Mục tiêu 1: So sánh Quy cách, Thông số, Model | Mục tiêu 2: Đánh giá mốc thời gian cơ sở đơn giá quá 12 tháng theo Quy định EVN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Mã ERP</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Tên Vật Tư Trình Duyệt</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>ĐVT</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Đơn Giá Trình (đ)</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>Thành Tiền Trình (đ)</t>
+        </is>
+      </c>
+      <c r="H4" s="61" t="inlineStr">
+        <is>
+          <t>Quy Cách, Model TRÌNH DUYỆT</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>Cơ Sở Đơn Giá Thẩm Định</t>
+        </is>
+      </c>
+      <c r="J4" s="61" t="inlineStr">
+        <is>
+          <t>Quy Cách, Model CƠ SỞ ĐƠN GIÁ</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>Đơn Giá Thống Nhất (đ)</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>Thành Tiền Thống Nhất (đ)</t>
+        </is>
+      </c>
+      <c r="M4" s="13" t="inlineStr">
+        <is>
+          <t>Giá Trị Giảm (đ)</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>% Giảm</t>
+        </is>
+      </c>
+      <c r="O4" s="61" t="inlineStr">
+        <is>
+          <t>[MỤC TIÊU 1] Đánh Giá Quy Cách &amp; Model</t>
+        </is>
+      </c>
+      <c r="P4" s="62" t="inlineStr">
+        <is>
+          <t>Số HĐ / Báo Giá / Quyết Định Cơ Sở</t>
+        </is>
+      </c>
+      <c r="Q4" s="62" t="inlineStr">
+        <is>
+          <t>Ngày Cơ Sở Đơn Giá</t>
+        </is>
+      </c>
+      <c r="R4" s="62" t="inlineStr">
+        <is>
+          <t>Ngày Thẩm Định</t>
+        </is>
+      </c>
+      <c r="S4" s="62" t="inlineStr">
+        <is>
+          <t>Thời Gian (Tháng)</t>
+        </is>
+      </c>
+      <c r="T4" s="62" t="inlineStr">
+        <is>
+          <t>[MỤC TIÊU 2] Đánh Giá Hiệu Lực (Mốc 12T)</t>
+        </is>
+      </c>
+      <c r="U4" s="13" t="inlineStr">
+        <is>
+          <t>Ghi Chú &amp; Thuyết Minh Thẩm Định</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Chưa có mã vật tư</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>Thanh cái đồng V phân phối mạ bạc</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>Thanh</t>
+        </is>
+      </c>
+      <c r="E5" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>48000000</v>
+      </c>
+      <c r="G5" s="27" t="n">
+        <v>192000000</v>
+      </c>
+      <c r="H5" s="26" t="inlineStr">
+        <is>
+          <t>Thanh cái đồng V phân phối mạ bạc
+Kích thước: 28x40x6mm
+Chiều dài: 920mm - Hãng: Kungho/ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="I5" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 2: CSDL ERP Vĩnh Tân 4</t>
+        </is>
+      </c>
+      <c r="J5" s="26" t="inlineStr">
+        <is>
+          <t>Thanh đồng mạ niken, KT: 30x600x5mm | Thanh đồng mạ niken, KT: 30x600x5mm</t>
+        </is>
+      </c>
+      <c r="K5" s="27" t="n">
+        <v>1390909</v>
+      </c>
+      <c r="L5" s="27" t="n">
+        <v>5563636</v>
+      </c>
+      <c r="M5" s="64" t="n">
+        <v>186436364</v>
+      </c>
+      <c r="N5" s="65" t="n">
+        <v>97.10227291666666</v>
+      </c>
+      <c r="O5" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P5" s="26" t="inlineStr">
+        <is>
+          <t>Nhập kho vật tư (HĐ:227) theo hóa đơn số 0000035 ngày 15.01.2021</t>
+        </is>
+      </c>
+      <c r="Q5" s="24" t="inlineStr">
+        <is>
+          <t>25/01/2021</t>
+        </is>
+      </c>
+      <c r="R5" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S5" s="24" t="n">
+        <v>68</v>
+      </c>
+      <c r="T5" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (68 tháng - 5.7 năm)</t>
+        </is>
+      </c>
+      <c r="U5" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 1,390,909 đ (giảm trừ 46,609,091 đ/đơn vị) căn cứ theo Cơ sở 2: CSDL ERP Vĩnh Tân 4, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Kungho/ Trung Quốc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Chưa có mã vật tư</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Công tơ nước dạng cơ, kích thước DN125</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>Cái</t>
+        </is>
+      </c>
+      <c r="E6" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="27" t="n">
+        <v>9660000</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>19320000</v>
+      </c>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>Công tơ nước dạng cơ, kích thước DN125, 8 lỗ bulong Ø16 ở mỗi đầu bích;
+Vật liệu: Cast iron;
+Môi chất làm việc: nước sạch (nước khử khoáng);
+Công tơ có giấy chứng nhận hiệu chuẩn. - Hãng: Zenner/ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="I6" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 3: EVN IMIS</t>
+        </is>
+      </c>
+      <c r="J6" s="26" t="inlineStr">
+        <is>
+          <t>Khớp nối mềm; SREJ-0125-16-D2R; DN125mm; PN16bar | Đơn vị: Công ty Thủy điện Buôn Kuốp</t>
+        </is>
+      </c>
+      <c r="K6" s="27" t="n">
+        <v>1972455</v>
+      </c>
+      <c r="L6" s="27" t="n">
+        <v>3944910</v>
+      </c>
+      <c r="M6" s="64" t="n">
+        <v>15375090</v>
+      </c>
+      <c r="N6" s="65" t="n">
+        <v>79.58121118012423</v>
+      </c>
+      <c r="O6" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P6" s="26" t="inlineStr">
+        <is>
+          <t>2603/2025/VTN_15</t>
+        </is>
+      </c>
+      <c r="Q6" s="24" t="inlineStr">
+        <is>
+          <t>26/03/2025</t>
+        </is>
+      </c>
+      <c r="R6" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S6" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="T6" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (18 tháng - 1.5 năm)</t>
+        </is>
+      </c>
+      <c r="U6" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 1,972,455 đ (giảm trừ 7,687,545 đ/đơn vị) căn cứ theo Cơ sở 3: EVN IMIS, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (DN125 - Zenner/ Trung Quốc). LÝ DO KỸ THUẬT KHÔNG ÁP D</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>5.05.65.658.KOR.00.000</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>Collector (chổi tiếp điện từ thanh ray)</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>Bộ</t>
+        </is>
+      </c>
+      <c r="E7" s="63" t="n">
+        <v>36</v>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>2265000</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <v>81540000</v>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>Collector (chổi tiếp điện từ thanh ray):
+- Iđm: 60A;
+- Uđm: 400VAC;
+- Material: Copper
+- Maker: Eunchang T&amp;C - Hãng: Eunchang/ Hàn Quốc</t>
+        </is>
+      </c>
+      <c r="I7" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 4: Mua Sắm Công e-GP</t>
+        </is>
+      </c>
+      <c r="J7" s="26" t="inlineStr">
+        <is>
+          <t>Chổi tiếp điện từ thanh ray (Electric collector); 60A; 400VAC.</t>
+        </is>
+      </c>
+      <c r="K7" s="27" t="n">
+        <v>1750000</v>
+      </c>
+      <c r="L7" s="27" t="n">
+        <v>63000000</v>
+      </c>
+      <c r="M7" s="64" t="n">
+        <v>18540000</v>
+      </c>
+      <c r="N7" s="65" t="n">
+        <v>22.73730684326711</v>
+      </c>
+      <c r="O7" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P7" s="26" t="inlineStr">
+        <is>
+          <t>IB2600422382</t>
+        </is>
+      </c>
+      <c r="Q7" s="24" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="R7" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S7" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T7" s="68" t="inlineStr">
+        <is>
+          <t>🟢 Trong hạn 12 tháng (0 tháng)</t>
+        </is>
+      </c>
+      <c r="U7" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 1,750,000 đ (giảm trừ 515,000 đ/đơn vị) căn cứ theo Cơ sở 4: Mua Sắm Công e-GP, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Eunchang/ Hàn Quốc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>4.90.80.030.KOR.00.000</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Bao che giữa các khớp nối đường ray cáp điện (Joint cover)</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>Cái</t>
+        </is>
+      </c>
+      <c r="E8" s="63" t="n">
+        <v>235</v>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>66000</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>15510000</v>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>Joint cover (bao che giữa các khớp nối đường ray cáp điện):
+- Material: PVC
+- Maker: Eunchang T&amp;C - Hãng: Eunchang/ Hàn Quốc</t>
+        </is>
+      </c>
+      <c r="I8" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 4: Mua Sắm Công e-GP</t>
+        </is>
+      </c>
+      <c r="J8" s="26" t="inlineStr">
+        <is>
+          <t>Bao che giữa các khớp nối đường ray cáp điện (Joint cover)</t>
+        </is>
+      </c>
+      <c r="K8" s="27" t="n">
+        <v>57000</v>
+      </c>
+      <c r="L8" s="27" t="n">
+        <v>13395000</v>
+      </c>
+      <c r="M8" s="64" t="n">
+        <v>2115000</v>
+      </c>
+      <c r="N8" s="65" t="n">
+        <v>13.63636363636363</v>
+      </c>
+      <c r="O8" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P8" s="26" t="inlineStr">
+        <is>
+          <t>IB2600422382</t>
+        </is>
+      </c>
+      <c r="Q8" s="24" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="R8" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S8" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T8" s="68" t="inlineStr">
+        <is>
+          <t>🟢 Trong hạn 12 tháng (0 tháng)</t>
+        </is>
+      </c>
+      <c r="U8" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 57,000 đ (giảm trừ 9,000 đ/đơn vị) căn cứ theo Cơ sở 4: Mua Sắm Công e-GP, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Eunchang/ Hàn Quốc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>4.90.80.027.KOR.00.000</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Nắp che phía cuối đường ray cáp điện (End cap)</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>Cái</t>
+        </is>
+      </c>
+      <c r="E9" s="63" t="n">
+        <v>32</v>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>68000</v>
+      </c>
+      <c r="G9" s="27" t="n">
+        <v>2176000</v>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>Nắp che phía cuối đường ray cáp điện (End cap)- Material: PVC
+- Maker: Eunchang T&amp;C - Hãng: Eunchang/ Hàn Quốc</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 2: CSDL ERP Vĩnh Tân 4</t>
+        </is>
+      </c>
+      <c r="J9" s="26" t="inlineStr">
+        <is>
+          <t>Bao che giữa các khớp nối đường ray cáp điện (Joint cover) | Bao che giữa các khớp nối đường ray cáp điện (Joint cover)</t>
+        </is>
+      </c>
+      <c r="K9" s="27" t="n">
+        <v>26000</v>
+      </c>
+      <c r="L9" s="27" t="n">
+        <v>832000</v>
+      </c>
+      <c r="M9" s="64" t="n">
+        <v>1344000</v>
+      </c>
+      <c r="N9" s="65" t="n">
+        <v>61.76470588235294</v>
+      </c>
+      <c r="O9" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P9" s="26" t="inlineStr">
+        <is>
+          <t>Nhập kho vật tư (HĐ:116/2022) theo hóa đơn số 00000008 ngày 27.02.2023</t>
+        </is>
+      </c>
+      <c r="Q9" s="24" t="inlineStr">
+        <is>
+          <t>27/02/2023</t>
+        </is>
+      </c>
+      <c r="R9" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S9" s="24" t="n">
+        <v>43</v>
+      </c>
+      <c r="T9" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (43 tháng - 3.6 năm)</t>
+        </is>
+      </c>
+      <c r="U9" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 26,000 đ (giảm trừ 42,000 đ/đơn vị) căn cứ theo Cơ sở 2: CSDL ERP Vĩnh Tân 4, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Eunchang/ Hàn Quốc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>2.08.37.001.KOR.97.000</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Trolley-bar (thanh ray cấp nguồn)</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>Cây</t>
+        </is>
+      </c>
+      <c r="E10" s="63" t="n">
+        <v>28</v>
+      </c>
+      <c r="F10" s="27" t="n">
+        <v>909000</v>
+      </c>
+      <c r="G10" s="27" t="n">
+        <v>25452000</v>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>Trolley-bar (thanh ray cấp nguồn):
+- Iđm: 60A;
+- Uđm: 400VAC;
+- Length: 3m / cây
+- Material: Copper
+- Maker: EunchangT&amp;C - Hãng: Eunchang/ Hàn Quốc</t>
+        </is>
+      </c>
+      <c r="I10" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 2: CSDL ERP Vĩnh Tân 4</t>
+        </is>
+      </c>
+      <c r="J10" s="26" t="inlineStr">
+        <is>
+          <t>Nắp che phía cuối đường ray cáp điện (End cap) | Nắp che phía cuối đường ray cáp điện (End cap)</t>
+        </is>
+      </c>
+      <c r="K10" s="27" t="n">
+        <v>21000</v>
+      </c>
+      <c r="L10" s="27" t="n">
+        <v>588000</v>
+      </c>
+      <c r="M10" s="64" t="n">
+        <v>24864000</v>
+      </c>
+      <c r="N10" s="65" t="n">
+        <v>97.6897689768977</v>
+      </c>
+      <c r="O10" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P10" s="26" t="inlineStr">
+        <is>
+          <t>Nhập kho vật tư (HĐ:116/2022) theo hóa đơn số 00000008 ngày 27.02.2023</t>
+        </is>
+      </c>
+      <c r="Q10" s="24" t="inlineStr">
+        <is>
+          <t>27/02/2023</t>
+        </is>
+      </c>
+      <c r="R10" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S10" s="24" t="n">
+        <v>43</v>
+      </c>
+      <c r="T10" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (43 tháng - 3.6 năm)</t>
+        </is>
+      </c>
+      <c r="U10" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 21,000 đ (giảm trừ 888,000 đ/đơn vị) căn cứ theo Cơ sở 2: CSDL ERP Vĩnh Tân 4, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Eunchang/ Hàn Quốc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Chưa có mã vật tư</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Lưỡi gà móc cẩu 3 tấn</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>Cái</t>
+        </is>
+      </c>
+      <c r="E11" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="27" t="n">
+        <v>610000</v>
+      </c>
+      <c r="G11" s="27" t="n">
+        <v>610000</v>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>Lưỡi gà móc cẩu 3 tấn
+Kích thước: rộng 25mm x dài 60mm - Hãng: MT/ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 2: CSDL ERP Vĩnh Tân 4</t>
+        </is>
+      </c>
+      <c r="J11" s="26" t="inlineStr">
+        <is>
+          <t>Lưỡi gà móc cẩu BCD10t, Kích thước (DxR): 120mmx41mm | Lưỡi gà móc cẩu BCD10t, Kích thước (DxR): 120mmx41mm</t>
+        </is>
+      </c>
+      <c r="K11" s="27" t="n">
+        <v>585000</v>
+      </c>
+      <c r="L11" s="27" t="n">
+        <v>585000</v>
+      </c>
+      <c r="M11" s="64" t="n">
+        <v>25000</v>
+      </c>
+      <c r="N11" s="65" t="n">
+        <v>4.098360655737705</v>
+      </c>
+      <c r="O11" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P11" s="26" t="inlineStr">
+        <is>
+          <t>Nhập kho vật tư (HĐ: 57/2024) theo hóa đơn số 615 ngày 27.08.2024</t>
+        </is>
+      </c>
+      <c r="Q11" s="24" t="inlineStr">
+        <is>
+          <t>06/09/2024</t>
+        </is>
+      </c>
+      <c r="R11" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S11" s="24" t="n">
+        <v>24</v>
+      </c>
+      <c r="T11" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (24 tháng - 2.0 năm)</t>
+        </is>
+      </c>
+      <c r="U11" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 585,000 đ (giảm trừ 25,000 đ/đơn vị) căn cứ theo Cơ sở 2: CSDL ERP Vĩnh Tân 4, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - MT/ Trung Quốc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>3.15.44.076.CHN.00.000</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Cáp điện dẹt cho cầu trục
+Quy cách: 16mm2 x 4C
+Ruột mềm</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>Mét</t>
+        </is>
+      </c>
+      <c r="E12" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="F12" s="27" t="n">
+        <v>711000</v>
+      </c>
+      <c r="G12" s="27" t="n">
+        <v>35550000</v>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>Cáp điện dẹt cho cầu trục
+Quy cách: 16mm2 x 4C
+Ruột mềm
+Điện áp: 450/750V
+Cách điện: PVC, dẻo
+NSX: Imatek - Hãng: Imatek/ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="I12" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 2: CSDL ERP Vĩnh Tân 4</t>
+        </is>
+      </c>
+      <c r="J12" s="26" t="inlineStr">
+        <is>
+          <t>Ống nối cáp điện; model: SL16, chất liệu đồng thau, tiết diện cáp sử dụng 16 mm2 | Ống nối cáp điện; model: SL16, chất liệu đồng thau, tiết diện cáp sử dụng 16 mm2</t>
+        </is>
+      </c>
+      <c r="K12" s="27" t="n">
+        <v>66000</v>
+      </c>
+      <c r="L12" s="27" t="n">
+        <v>3300000</v>
+      </c>
+      <c r="M12" s="64" t="n">
+        <v>32250000</v>
+      </c>
+      <c r="N12" s="65" t="n">
+        <v>90.71729957805907</v>
+      </c>
+      <c r="O12" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P12" s="26" t="inlineStr">
+        <is>
+          <t>Nhập kho vật tư (HĐ: 113/2025) theo hóa đơn số 00000004 ngày 08.01.2026</t>
+        </is>
+      </c>
+      <c r="Q12" s="24" t="inlineStr">
+        <is>
+          <t>23/01/2026</t>
+        </is>
+      </c>
+      <c r="R12" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S12" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="T12" s="68" t="inlineStr">
+        <is>
+          <t>🟢 Trong hạn 12 tháng (8 tháng)</t>
+        </is>
+      </c>
+      <c r="U12" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 66,000 đ (giảm trừ 645,000 đ/đơn vị) căn cứ theo Cơ sở 2: CSDL ERP Vĩnh Tân 4, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Imatek/ Trung Quốc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>3.20.22.003.TPE.00.000</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Khóa cáp 
+Dùng cho cáp: 3mm</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>Cái</t>
+        </is>
+      </c>
+      <c r="E13" s="63" t="n">
+        <v>55</v>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>14000</v>
+      </c>
+      <c r="G13" s="27" t="n">
+        <v>770000</v>
+      </c>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>Khóa cáp 
+Dùng cho cáp: 3mm - Hãng: Kungho/ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 4: Mua Sắm Công e-GP</t>
+        </is>
+      </c>
+      <c r="J13" s="26" t="inlineStr">
+        <is>
+          <t>Khóa cáp 4</t>
+        </is>
+      </c>
+      <c r="K13" s="27" t="n">
+        <v>1852</v>
+      </c>
+      <c r="L13" s="27" t="n">
+        <v>101860</v>
+      </c>
+      <c r="M13" s="64" t="n">
+        <v>668140</v>
+      </c>
+      <c r="N13" s="65" t="n">
+        <v>86.77142857142857</v>
+      </c>
+      <c r="O13" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P13" s="26" t="inlineStr">
+        <is>
+          <t>IB2600528351</t>
+        </is>
+      </c>
+      <c r="Q13" s="24" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="R13" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S13" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T13" s="68" t="inlineStr">
+        <is>
+          <t>🟢 Trong hạn 12 tháng (0 tháng)</t>
+        </is>
+      </c>
+      <c r="U13" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 1,852 đ (giảm trừ 12,148 đ/đơn vị) căn cứ theo Cơ sở 4: Mua Sắm Công e-GP, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Kungho/ Trung Quốc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>5.01.07.302.FRA.00.000</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Bạc đạn 6302</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>Cái</t>
+        </is>
+      </c>
+      <c r="E14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="27" t="n">
+        <v>158000</v>
+      </c>
+      <c r="G14" s="27" t="n">
+        <v>316000</v>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>Bạc đạn 6302 - Hãng: SKF/ Pháp</t>
+        </is>
+      </c>
+      <c r="I14" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 4: Mua Sắm Công e-GP</t>
+        </is>
+      </c>
+      <c r="J14" s="26" t="inlineStr">
+        <is>
+          <t>Bạc đạn  6302 
+Các thông số cơ bản:
+- Tải trọng động: 11.9 kN;
+- Tải trọng tĩnh: 5.4 kN;
+- Vận tốc tham khảo: 38000 v/ph;
+- Vận tốc giới hạn: 24000 v/ph; 
+Nhà sản xuất/XX: SKF/China, Eu-G7</t>
+        </is>
+      </c>
+      <c r="K14" s="27" t="n">
+        <v>40560</v>
+      </c>
+      <c r="L14" s="27" t="n">
+        <v>81120</v>
+      </c>
+      <c r="M14" s="64" t="n">
+        <v>234880</v>
+      </c>
+      <c r="N14" s="65" t="n">
+        <v>74.32911392405063</v>
+      </c>
+      <c r="O14" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P14" s="26" t="inlineStr">
+        <is>
+          <t>IB2300309906</t>
+        </is>
+      </c>
+      <c r="Q14" s="24" t="inlineStr">
+        <is>
+          <t>27/12/2023</t>
+        </is>
+      </c>
+      <c r="R14" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S14" s="24" t="n">
+        <v>33</v>
+      </c>
+      <c r="T14" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (33 tháng - 2.8 năm)</t>
+        </is>
+      </c>
+      <c r="U14" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 40,560 đ (giảm trừ 117,440 đ/đơn vị) căn cứ theo Cơ sở 4: Mua Sắm Công e-GP, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - SKF/ Pháp).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Chưa có mã vật tư</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Bạc đạn 6208</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Vòng</t>
+        </is>
+      </c>
+      <c r="E15" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" s="27" t="n">
+        <v>444000</v>
+      </c>
+      <c r="G15" s="27" t="n">
+        <v>1776000</v>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>Bạc đạn 6208 - Hãng: SKF/ Pháp</t>
+        </is>
+      </c>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 2: CSDL ERP Vĩnh Tân 4</t>
+        </is>
+      </c>
+      <c r="J15" s="26" t="inlineStr">
+        <is>
+          <t>Bạc đạn 6302 | Bạc đạn 6302</t>
+        </is>
+      </c>
+      <c r="K15" s="27" t="n">
+        <v>85000</v>
+      </c>
+      <c r="L15" s="27" t="n">
+        <v>340000</v>
+      </c>
+      <c r="M15" s="64" t="n">
+        <v>1436000</v>
+      </c>
+      <c r="N15" s="65" t="n">
+        <v>80.85585585585585</v>
+      </c>
+      <c r="O15" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P15" s="26" t="inlineStr">
+        <is>
+          <t>Nhập kho Bạc đạn (HĐ:223) theo hóa đơn số 0000792 ngày 31.12.2020 (phiếu sai)</t>
+        </is>
+      </c>
+      <c r="Q15" s="24" t="inlineStr">
+        <is>
+          <t>19/01/2021</t>
+        </is>
+      </c>
+      <c r="R15" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S15" s="24" t="n">
+        <v>68</v>
+      </c>
+      <c r="T15" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (68 tháng - 5.7 năm)</t>
+        </is>
+      </c>
+      <c r="U15" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 85,000 đ (giảm trừ 359,000 đ/đơn vị) căn cứ theo Cơ sở 2: CSDL ERP Vĩnh Tân 4, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - SKF/ Pháp).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Chưa có mã vật tư</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Keo phủ chống mài mòn Kalpoxy-150</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>Cặp</t>
+        </is>
+      </c>
+      <c r="E16" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="F16" s="27" t="n">
+        <v>16320000</v>
+      </c>
+      <c r="G16" s="27" t="n">
+        <v>326400000</v>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>Wear Resistant Mortar (Keo chống mài mòn)
+Keo phủ chống mài mòn Kalpoxy-150/Kalenborn 
+(01 cặp bao gồm hardener + Resin) - Hãng: Kalenborn/ Đức</t>
+        </is>
+      </c>
+      <c r="I16" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 4: Mua Sắm Công e-GP</t>
+        </is>
+      </c>
+      <c r="J16" s="26" t="inlineStr">
+        <is>
+          <t>Keo phủ chống mài mòn</t>
+        </is>
+      </c>
+      <c r="K16" s="27" t="n">
+        <v>1596000</v>
+      </c>
+      <c r="L16" s="27" t="n">
+        <v>31920000</v>
+      </c>
+      <c r="M16" s="64" t="n">
+        <v>294480000</v>
+      </c>
+      <c r="N16" s="65" t="n">
+        <v>90.22058823529412</v>
+      </c>
+      <c r="O16" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P16" s="26" t="inlineStr">
+        <is>
+          <t>IB2500075655</t>
+        </is>
+      </c>
+      <c r="Q16" s="24" t="inlineStr">
+        <is>
+          <t>11/05/2025</t>
+        </is>
+      </c>
+      <c r="R16" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S16" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="T16" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (16 tháng - 1.3 năm)</t>
+        </is>
+      </c>
+      <c r="U16" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 1,596,000 đ (giảm trừ 14,724,000 đ/đơn vị) căn cứ theo Cơ sở 4: Mua Sắm Công e-GP, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Kalenborn/ Đức).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>3.70.75.349.CHN.99.000</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Cao su non, KT: B500x6x2800mm</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>Cuộn</t>
+        </is>
+      </c>
+      <c r="E17" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="F17" s="27" t="n">
+        <v>6200000</v>
+      </c>
+      <c r="G17" s="27" t="n">
+        <v>124000000</v>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>Cao su non, KT: B500x6x2800mm - Hãng: Rema Tiptop/ Đức</t>
+        </is>
+      </c>
+      <c r="I17" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 4: Mua Sắm Công e-GP</t>
+        </is>
+      </c>
+      <c r="J17" s="26" t="inlineStr">
+        <is>
+          <t>Cao su non; KT B500x6x2800mm; Mã 538 0048
+NSX: Rema TipTop</t>
+        </is>
+      </c>
+      <c r="K17" s="27" t="n">
+        <v>4881000</v>
+      </c>
+      <c r="L17" s="27" t="n">
+        <v>97620000</v>
+      </c>
+      <c r="M17" s="64" t="n">
+        <v>26380000</v>
+      </c>
+      <c r="N17" s="65" t="n">
+        <v>21.2741935483871</v>
+      </c>
+      <c r="O17" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P17" s="26" t="inlineStr">
+        <is>
+          <t>IB2300253768</t>
+        </is>
+      </c>
+      <c r="Q17" s="24" t="inlineStr">
+        <is>
+          <t>30/11/2023</t>
+        </is>
+      </c>
+      <c r="R17" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S17" s="24" t="n">
+        <v>34</v>
+      </c>
+      <c r="T17" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (34 tháng - 2.8 năm)</t>
+        </is>
+      </c>
+      <c r="U17" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 4,881,000 đ (giảm trừ 1,319,000 đ/đơn vị) căn cứ theo Cơ sở 4: Mua Sắm Công e-GP, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Rema Tiptop/ Đức).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>Chưa có mã vật tư</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Bản quyền Windows 11 Pro</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>License</t>
+        </is>
+      </c>
+      <c r="E18" s="63" t="n">
+        <v>123</v>
+      </c>
+      <c r="F18" s="27" t="n">
+        <v>5300000</v>
+      </c>
+      <c r="G18" s="27" t="n">
+        <v>651900000</v>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>Windows GGWA - Windows 11 Pro - Legalization Get Genuine - Hãng: Microsoft/ USA</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 3: EVN IMIS</t>
+        </is>
+      </c>
+      <c r="J18" s="26" t="inlineStr">
+        <is>
+          <t>Phần mềm Bản quyền Windows 11 Pro, Thời hạn bản quyền: vĩnh viễn | Đơn vị: Công ty Nhiệt điện Duyên Hải</t>
+        </is>
+      </c>
+      <c r="K18" s="27" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="L18" s="27" t="n">
+        <v>553500000</v>
+      </c>
+      <c r="M18" s="64" t="n">
+        <v>98400000</v>
+      </c>
+      <c r="N18" s="65" t="n">
+        <v>15.09433962264151</v>
+      </c>
+      <c r="O18" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P18" s="26" t="inlineStr">
+        <is>
+          <t>134.23/DTG</t>
+        </is>
+      </c>
+      <c r="Q18" s="24" t="inlineStr">
+        <is>
+          <t>21/12/2023</t>
+        </is>
+      </c>
+      <c r="R18" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S18" s="24" t="n">
+        <v>33</v>
+      </c>
+      <c r="T18" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (33 tháng - 2.8 năm)</t>
+        </is>
+      </c>
+      <c r="U18" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 4,500,000 đ (giảm trừ 800,000 đ/đơn vị) căn cứ theo Cơ sở 3: EVN IMIS, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (WINDOWS 11 - Microsoft/ USA). LÝ DO KỸ THUẬT KHÔNG ÁP DỤ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>Chưa có mã vật tư</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Động cơ và bơm NAOH, Type: TP400 PP, FCA 112 MC-2/HE, Công suất: 5,5kW</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>Bộ</t>
+        </is>
+      </c>
+      <c r="E19" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="27" t="n">
+        <v>770000000</v>
+      </c>
+      <c r="G19" s="27" t="n">
+        <v>1540000000</v>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>Bơm (SP-Circulation pump):
+TP400 PP, P4-400V/50
+Động cơ bơm: type: FCA 112 MC-2/PHE, Công Suất : 5,5kW
+Điện áp: 400Vac
+Tần số: 50Hz
+Dòng định mức: 10.11A,
+Tốc độ quay: 2900 rpm
+Trọng lượng: 34kg
+Poles: 2P, Insulation class: F
+Degress of protection: IP55,
+PF: 0,88, Connection: Sao /Tam giác (400/690 YV), Eff: 0,87 - 0,89
+Standard Specification :
+IEC60034-1 - Hãng: Grundfos/ Eu</t>
+        </is>
+      </c>
+      <c r="I19" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 1: Báo giá cạnh tranh</t>
+        </is>
+      </c>
+      <c r="J19" s="26" t="inlineStr">
+        <is>
+          <t>Báo giá cạnh tranh nộp kèm đợt thẩm định 2026</t>
+        </is>
+      </c>
+      <c r="K19" s="27" t="n">
+        <v>750000000</v>
+      </c>
+      <c r="L19" s="27" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="M19" s="64" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="N19" s="65" t="n">
+        <v>2.597402597402597</v>
+      </c>
+      <c r="O19" s="66" t="inlineStr">
+        <is>
+          <t>✅ Báo giá cạnh tranh đáp ứng 100% hồ sơ yêu cầu kỹ thuật</t>
+        </is>
+      </c>
+      <c r="P19" s="26" t="inlineStr">
+        <is>
+          <t>Báo giá NCC chào cạnh tranh</t>
+        </is>
+      </c>
+      <c r="Q19" s="24" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="R19" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S19" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T19" s="68" t="inlineStr">
+        <is>
+          <t>🟢 Trong hạn 12 tháng (0 tháng)</t>
+        </is>
+      </c>
+      <c r="U19" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 750,000,000 đ (giảm trừ 20,000,000 đ/đơn vị) căn cứ theo Cơ sở 1: Báo giá cạnh tranh, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (TP400 - Grundfos/ Eu). LÝ DO KỸ THUẬT KHÔ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>5.33.85.051.CHN.00.000</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Phanh đuôi động cơ, model: BFK458-18E</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>Bộ</t>
+        </is>
+      </c>
+      <c r="E20" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="27" t="n">
+        <v>63063000</v>
+      </c>
+      <c r="G20" s="27" t="n">
+        <v>126126000</v>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>Model: BFK458-18E
+Size: 18
+Đường kính phủ bì: 218,6mm
+Lỗ lắp bulong: 6xM8
+Đường kính vòng chia bulong: 196mm
+Điện áp: 205VDC
+Nhà sản xuất: INTORQ - Hãng: Intorq/ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 3: EVN IMIS</t>
+        </is>
+      </c>
+      <c r="J20" s="26" t="inlineStr">
+        <is>
+          <t>Phanh xe lớn Loại BFK458-16E | Đơn vị: Công ty Cổ phần Thủy điện Sông Ba Hạ</t>
+        </is>
+      </c>
+      <c r="K20" s="27" t="n">
+        <v>30380000</v>
+      </c>
+      <c r="L20" s="27" t="n">
+        <v>60760000</v>
+      </c>
+      <c r="M20" s="64" t="n">
+        <v>65366000</v>
+      </c>
+      <c r="N20" s="65" t="n">
+        <v>51.82595182595182</v>
+      </c>
+      <c r="O20" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P20" s="26" t="inlineStr">
+        <is>
+          <t>30/HĐ-SBH</t>
+        </is>
+      </c>
+      <c r="Q20" s="24" t="inlineStr">
+        <is>
+          <t>17/05/2024</t>
+        </is>
+      </c>
+      <c r="R20" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S20" s="24" t="n">
+        <v>28</v>
+      </c>
+      <c r="T20" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (28 tháng - 2.3 năm)</t>
+        </is>
+      </c>
+      <c r="U20" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 30,380,000 đ (giảm trừ 32,683,000 đ/đơn vị) căn cứ theo Cơ sở 3: EVN IMIS, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (BFK458-18E - Intorq/ Trung Quốc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>1.31.23.425.CHN.00.000</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Nhớt SHELL OMALA S4 WE 220</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>Lít</t>
+        </is>
+      </c>
+      <c r="E21" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="F21" s="27" t="n">
+        <v>560000</v>
+      </c>
+      <c r="G21" s="27" t="n">
+        <v>11200000</v>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>Nhớt SHELL OMALA S4 WE 220; Độ nhớt ISO VG 220; Qui cách: 20l/xô; NSX: Shell/tương đương - Hãng: Shell/ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="I21" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 3: EVN IMIS</t>
+        </is>
+      </c>
+      <c r="J21" s="26" t="inlineStr">
+        <is>
+          <t>Dầu hộp số Shell Omala S4 WE 220 | Đơn vị: EVN - Công ty Nhiệt điện Thái Bình</t>
+        </is>
+      </c>
+      <c r="K21" s="27" t="n">
+        <v>347000</v>
+      </c>
+      <c r="L21" s="27" t="n">
+        <v>6940000</v>
+      </c>
+      <c r="M21" s="64" t="n">
+        <v>4260000</v>
+      </c>
+      <c r="N21" s="65" t="n">
+        <v>38.03571428571428</v>
+      </c>
+      <c r="O21" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P21" s="26" t="inlineStr">
+        <is>
+          <t>72/HĐ-HH04-2023</t>
+        </is>
+      </c>
+      <c r="Q21" s="24" t="inlineStr">
+        <is>
+          <t>01/08/2023</t>
+        </is>
+      </c>
+      <c r="R21" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S21" s="24" t="n">
+        <v>37</v>
+      </c>
+      <c r="T21" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (37 tháng - 3.1 năm)</t>
+        </is>
+      </c>
+      <c r="U21" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đơn giá đề nghị 347,000 đ (giảm trừ 213,000 đ/đơn vị) căn cứ theo Cơ sở 3: EVN IMIS, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (WE 220 - Shell/ Trung Quốc). LÝ DO KỸ THUẬT KHÔNG ÁP DỤNG </t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>5.30.10.355.VIE.99.000</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Gàu múc MĐPĐ, Thể tích: 0.75m3, Vật liệu: E355DD</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>cái</t>
+        </is>
+      </c>
+      <c r="E22" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="27" t="n">
+        <v>265000000</v>
+      </c>
+      <c r="G22" s="27" t="n">
+        <v>530000000</v>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>Gàu múc MĐPĐ, Thể tích: 0.75m3, Vật liệu: E355DD - Hãng: Việt Nam</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>Cơ sở 2: CSDL ERP Vĩnh Tân 4</t>
+        </is>
+      </c>
+      <c r="J22" s="26" t="inlineStr">
+        <is>
+          <t>Gầu múc ĐPĐ, thể tích 0.75m3, vật liệu: SMS570(JIS)+A709(ASTM) | Gầu múc ĐPĐ, thể tích 0.75m3, vật liệu: SMS570(JIS)+A709(ASTM)</t>
+        </is>
+      </c>
+      <c r="K22" s="27" t="n">
+        <v>137382000</v>
+      </c>
+      <c r="L22" s="27" t="n">
+        <v>274764000</v>
+      </c>
+      <c r="M22" s="64" t="n">
+        <v>255236000</v>
+      </c>
+      <c r="N22" s="65" t="n">
+        <v>48.15773584905661</v>
+      </c>
+      <c r="O22" s="66" t="inlineStr">
+        <is>
+          <t>✅ Khớp đúng Model &amp; Thông số kỹ thuật yêu cầu</t>
+        </is>
+      </c>
+      <c r="P22" s="26" t="inlineStr">
+        <is>
+          <t>Nhập kho vật tư (HĐ: 63/2024) theo hóa đơn số 37 ngày 22.10.2024</t>
+        </is>
+      </c>
+      <c r="Q22" s="24" t="inlineStr">
+        <is>
+          <t>04/11/2024</t>
+        </is>
+      </c>
+      <c r="R22" s="24" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="S22" s="24" t="n">
+        <v>22</v>
+      </c>
+      <c r="T22" s="67" t="inlineStr">
+        <is>
+          <t>🟡 Quá 12 tháng (22 tháng - 1.8 năm)</t>
+        </is>
+      </c>
+      <c r="U22" s="26" t="inlineStr">
+        <is>
+          <t>Đơn giá đề nghị 137,382,000 đ (giảm trừ 127,618,000 đ/đơn vị) căn cứ theo Cơ sở 2: CSDL ERP Vĩnh Tân 4, bảo đảm trùng khớp chính xác thông số kỹ thuật và Model (Theo thiết kế - Việt Nam).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG (18 MỤC TIẾT GIẢM):</t>
+        </is>
+      </c>
+      <c r="B23" s="50" t="n"/>
+      <c r="C23" s="50" t="n"/>
+      <c r="D23" s="50" t="n"/>
+      <c r="E23" s="50" t="n"/>
+      <c r="F23" s="50" t="n"/>
+      <c r="G23" s="51" t="n">
+        <v>3684646000</v>
+      </c>
+      <c r="H23" s="50" t="n"/>
+      <c r="I23" s="50" t="n"/>
+      <c r="J23" s="50" t="n"/>
+      <c r="K23" s="50" t="n"/>
+      <c r="L23" s="51" t="n">
+        <v>2617235526</v>
+      </c>
+      <c r="M23" s="52" t="n">
+        <v>1067410474</v>
+      </c>
+      <c r="N23" s="69" t="n">
+        <v>28.9691458555313</v>
+      </c>
+      <c r="O23" s="50" t="n"/>
+      <c r="P23" s="50" t="n"/>
+      <c r="Q23" s="50" t="n"/>
+      <c r="R23" s="50" t="n"/>
+      <c r="S23" s="50" t="n"/>
+      <c r="T23" s="50" t="n"/>
+      <c r="U23" s="50" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>